<commit_message>
Atualiza historico e planilhas PICKUP (run automatico)
</commit_message>
<xml_diff>
--- a/output/PICKUP_diario.xlsx
+++ b/output/PICKUP_diario.xlsx
@@ -542,7 +542,7 @@
         <v>0.9997</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.872</v>
+        <v>0.852</v>
       </c>
     </row>
     <row r="4">
@@ -572,7 +572,7 @@
         <v>0.9593</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.9390999999999999</v>
+        <v>0.9164</v>
       </c>
     </row>
     <row r="5">
@@ -626,7 +626,7 @@
         <v>0.9586</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.9904000000000001</v>
+        <v>0.9939</v>
       </c>
     </row>
     <row r="7">
@@ -656,7 +656,7 @@
         <v>0.9994</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0.5075</v>
+        <v>0.5276</v>
       </c>
     </row>
     <row r="8">
@@ -686,7 +686,7 @@
         <v>0.9947</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.9128000000000001</v>
+        <v>0.9029</v>
       </c>
     </row>
     <row r="9">
@@ -740,7 +740,7 @@
         <v>0.8826000000000001</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.9398000000000001</v>
+        <v>0.9451000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -824,7 +824,7 @@
         <v>0.9965999999999999</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.9235</v>
+        <v>0.9442</v>
       </c>
     </row>
     <row r="14">

</xml_diff>